<commit_message>
docs: adjust contribution ratios based on workload
- 代码+Solution (王, 周): 0.22 each (heaviest workload)
- PPT制作 (孙, 杨): 0.19 each
- PPT讲稿 (张): 0.18
</commit_message>
<xml_diff>
--- a/组内贡献分配表.xlsx
+++ b/组内贡献分配表.xlsx
@@ -547,7 +547,7 @@
         </is>
       </c>
       <c r="F2" s="4" t="n">
-        <v>0.25</v>
+        <v>0.22</v>
       </c>
     </row>
     <row r="3">
@@ -575,7 +575,7 @@
         </is>
       </c>
       <c r="F3" s="7" t="n">
-        <v>0.25</v>
+        <v>0.22</v>
       </c>
     </row>
     <row r="4">
@@ -603,7 +603,7 @@
         </is>
       </c>
       <c r="F4" s="4" t="n">
-        <v>0.2</v>
+        <v>0.19</v>
       </c>
     </row>
     <row r="5">
@@ -631,7 +631,7 @@
         </is>
       </c>
       <c r="F5" s="7" t="n">
-        <v>0.15</v>
+        <v>0.19</v>
       </c>
     </row>
     <row r="6">
@@ -659,7 +659,7 @@
         </is>
       </c>
       <c r="F6" s="4" t="n">
-        <v>0.15</v>
+        <v>0.18</v>
       </c>
     </row>
     <row r="7">

</xml_diff>